<commit_message>
added excel utils for doctor module
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -8,13 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2480269\Downloads\demo\mediconnect-automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E8CCDA-620B-4BA0-AD1B-843DDE258337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03DB0315-67C0-4FBC-B012-A56B4FF9B4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{20EC9760-B52E-4482-B97D-09277A4A575D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="8" activeTab="10" xr2:uid="{20EC9760-B52E-4482-B97D-09277A4A575D}"/>
   </bookViews>
   <sheets>
     <sheet name="Logins" sheetId="1" r:id="rId1"/>
     <sheet name="PatientRegister" sheetId="2" r:id="rId2"/>
+    <sheet name="AddPatient" sheetId="3" r:id="rId3"/>
+    <sheet name="NewAppointment" sheetId="4" r:id="rId4"/>
+    <sheet name="RequestLabTest" sheetId="5" r:id="rId5"/>
+    <sheet name="NewRecord" sheetId="6" r:id="rId6"/>
+    <sheet name="ScheduleSession" sheetId="7" r:id="rId7"/>
+    <sheet name="AddItem" sheetId="8" r:id="rId8"/>
+    <sheet name="AiAssistant" sheetId="9" r:id="rId9"/>
+    <sheet name="DoctorRegister" sheetId="10" r:id="rId10"/>
+    <sheet name="DoctorLogin" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="108">
   <si>
     <t>testId</t>
   </si>
@@ -96,6 +105,9 @@
     <t>TP001_patient_register</t>
   </si>
   <si>
+    <t>Auto</t>
+  </si>
+  <si>
     <t>Password@1</t>
   </si>
   <si>
@@ -175,13 +187,199 @@
   </si>
   <si>
     <t>Priya@9012</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>emergencyContact</t>
+  </si>
+  <si>
+    <t>DPA001_add_patient</t>
+  </si>
+  <si>
+    <t>auto_patient_${UNIQUE}@test.com</t>
+  </si>
+  <si>
+    <t>Patient@1234</t>
+  </si>
+  <si>
+    <t>Emergency - 8888888888</t>
+  </si>
+  <si>
+    <t>patientSearchQuery</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>DAP001_new_appointment</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>11:30AM</t>
+  </si>
+  <si>
+    <t>In-person</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>testType</t>
+  </si>
+  <si>
+    <t>priority</t>
+  </si>
+  <si>
+    <t>requestedDate</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>DLR001_request_test</t>
+  </si>
+  <si>
+    <t>CBC</t>
+  </si>
+  <si>
+    <t>Routine</t>
+  </si>
+  <si>
+    <t>Automated test request — please ignore</t>
+  </si>
+  <si>
+    <t>recordDate</t>
+  </si>
+  <si>
+    <t>diagnosis</t>
+  </si>
+  <si>
+    <t>treatment</t>
+  </si>
+  <si>
+    <t>prescription</t>
+  </si>
+  <si>
+    <t>clinicalNotes</t>
+  </si>
+  <si>
+    <t>DMR001_new_record</t>
+  </si>
+  <si>
+    <t>Automated test diagnosis - routine check</t>
+  </si>
+  <si>
+    <t>Rest, hydration, follow-up in 7 days</t>
+  </si>
+  <si>
+    <t>Paracetamol | 500mg | 1-0-1</t>
+  </si>
+  <si>
+    <t>Created by Selenium automation suite</t>
+  </si>
+  <si>
+    <t>duration</t>
+  </si>
+  <si>
+    <t>reason</t>
+  </si>
+  <si>
+    <t>DTM001_schedule_session</t>
+  </si>
+  <si>
+    <t>Automated test - follow up consultation</t>
+  </si>
+  <si>
+    <t>itemName</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>reorderLevel</t>
+  </si>
+  <si>
+    <t>DSC001_add_item</t>
+  </si>
+  <si>
+    <t>Paracetamol ${UNIQUE}</t>
+  </si>
+  <si>
+    <t>Medication</t>
+  </si>
+  <si>
+    <t>question</t>
+  </si>
+  <si>
+    <t>DAI001_normal_range</t>
+  </si>
+  <si>
+    <t>What is the normal range for HbA1c?</t>
+  </si>
+  <si>
+    <t>DAI002_drug_dose</t>
+  </si>
+  <si>
+    <t>Common side effects of Lisinopril</t>
+  </si>
+  <si>
+    <t>DAI003_lab_interpret</t>
+  </si>
+  <si>
+    <t>How to interpret a BNP result?</t>
+  </si>
+  <si>
+    <t>specialization</t>
+  </si>
+  <si>
+    <t>hospital</t>
+  </si>
+  <si>
+    <t>TD001_doctor_register</t>
+  </si>
+  <si>
+    <t>Doctor${UNIQUE}</t>
+  </si>
+  <si>
+    <t>auto.doctor.${UNIQUE}@test.com</t>
+  </si>
+  <si>
+    <t>Cardiology</t>
+  </si>
+  <si>
+    <t>Test Hospital</t>
+  </si>
+  <si>
+    <t>TC_DOC_LOGIN_VALID</t>
+  </si>
+  <si>
+    <t>arun.kumar@cgh.com</t>
+  </si>
+  <si>
+    <t>MediConnect@123</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,6 +397,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -263,24 +469,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -694,6 +901,115 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87715164-B4A9-4967-BE68-FEBD691217EB}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E2" s="8">
+        <v>9876543210</v>
+      </c>
+      <c r="F2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E80DC387-7ADE-42F2-AD04-E9AC427B8F77}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5547E1-8265-48F6-A84D-52EAF56CC962}">
   <dimension ref="A1:I5"/>
@@ -717,7 +1033,7 @@
         <v>12</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>1</v>
@@ -743,42 +1059,42 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>23</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>22</v>
       </c>
       <c r="E2" s="9">
         <v>9876543210</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G2" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>19</v>
-      </c>
-      <c r="I2" s="8" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" s="11">
         <v>9123456701</v>
@@ -787,27 +1103,27 @@
         <v>3121988</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E4" s="4">
         <v>9123456702</v>
@@ -816,27 +1132,27 @@
         <v>3121988</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E5" s="4">
         <v>9123456702</v>
@@ -845,13 +1161,13 @@
         <v>3121988</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -860,4 +1176,439 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E08C65E8-DE7E-42A4-B37E-94981247A45D}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="3.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="8">
+        <v>9999999999</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2">
+        <v>30</v>
+      </c>
+      <c r="H2" s="8">
+        <v>34700</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5BE7F55-1345-4108-923B-0A41576493AB}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="8">
+        <v>46188</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D9C8C5-C73D-486C-8F51-3D510C42F653}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="8">
+        <v>46188</v>
+      </c>
+      <c r="F2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FFAC5E4-BDFE-4DC7-B957-884FFA341B3B}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="8">
+        <v>46188</v>
+      </c>
+      <c r="D2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97E58940-03EA-43D5-AB8A-F1428AB480A3}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="8">
+        <v>46188</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2">
+        <v>30</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8D8907D-C1D4-4085-BA57-C8F8A8DB6768}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2">
+        <v>100</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1DC6E31-8F32-4B15-972B-7124E1050FED}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Changes with respect to data driven testing in patient
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -481,6 +481,9 @@
     <sheet name="SupplyOrders" sheetId="8" r:id="rId10"/>
     <sheet name="TelemedicineSessions" sheetId="9" r:id="rId11"/>
     <sheet name="AnalyticsFilters" sheetId="10" r:id="rId12"/>
+    <sheet name="PatientBookings" sheetId="11" r:id="rId13"/>
+    <sheet name="LabReportAIQuestions" sheetId="12" r:id="rId14"/>
+    <sheet name="AiAssistantInteractions" sheetId="13" r:id="rId15"/>
   </sheets>
   <calcPr fullPrecision="1" calcId="125725"/>
 </workbook>
@@ -749,6 +752,481 @@
       <c r="D6" t="inlineStr">
         <is>
           <t>Last 30 Days</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>testId</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>doctor</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TBA001_arun_inperson</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Dr. Arun Kumar — Cardiology</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Cardiology follow-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TBA002_meena_video</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dr. Meena Reddy — Neurology</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Neurology consultation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TBA003_vikram_inperson</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dr. Vikram Singh — Orthopedics</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2:00 PM</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Knee pain checkup</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>testId</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>question</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TQ001_chip_ldl</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>What is LDL cholesterol?</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>chip</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TQ002_chip_lower_ldl</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>How to lower LDL naturally?</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>chip</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TQ003_chip_statins</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>What are statins?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>chip</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TQ004_chip_ecg</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Is my ECG result good?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>chip</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TQ005_type_hdl</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>What does HDL mean?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TQ006_type_blood_test</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Explain my blood test results</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>testId</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TAH001_chip_lipid</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>General Chat</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>chip</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Explain my lipid panel results</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TAH002_chip_ldl</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>General Chat</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>chip</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>What does elevated LDL mean?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TAH003_type_cholesterol</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>General Chat</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>What are normal cholesterol levels?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TAH004_type_symptoms</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Symptom Checker</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>I have a headache and fever for 2 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TAH005_quick_symptom</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>quickAction</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Symptom Checker</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TAH006_quick_lab</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>quickAction</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Explain My Lab Report</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TAH007_common_bp</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>commonQuestion</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>What does my blood pressure reading mean?</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TAH008_common_diabetes</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>commonQuestion</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>How can I manage my diabetes better?</t>
         </is>
       </c>
     </row>

</xml_diff>